<commit_message>
Update blog post date to trigger build
</commit_message>
<xml_diff>
--- a/FSP_Blog_Competitive_Analysis.xlsx
+++ b/FSP_Blog_Competitive_Analysis.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Top FSP Blog Posts" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Topic Analysis" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Content Type Analysis" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="High Potential for FaMED" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Executive Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top FSP Blog Posts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topic Analysis" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Type Analysis" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Potential for FaMED" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1485,6 +1485,138 @@
       <c r="J21" s="4" t="inlineStr">
         <is>
           <t>FaMED Protokoll Book vs FaMED App: Which Investment is Better?</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>FSP Vokabelliste: 500 Essential Medical Terms</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Vocabulary</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>85</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>FaMED Essential Vocabulary: 500 Must-Know German Medical Terms</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>FSP Prüfung Bayern: Regional Differences Explained</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Regional Guide</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>72</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>FaMED State-by-State Guide: Regional Requirements in Germany</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>FSP Vokabelliste: 500 Essential Medical Terms</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Vocabulary</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>85</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>FaMED Essential Vocabulary: 500 Must-Know German Medical Terms</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>FSP Prüfung Bayern: Regional Differences Explained</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Regional Guide</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>72</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>FaMED State-by-State Guide: Regional Requirements in Germany</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Queued</t>
         </is>
       </c>
     </row>

</xml_diff>